<commit_message>
remove the season dropdown menu and replace with a persistent storage of selected season for only the count and the health page. change the loctile so that the hard code take in the size of the reconstructed image
</commit_message>
<xml_diff>
--- a/docs/AIMS_Tiles_Columns.xlsx
+++ b/docs/AIMS_Tiles_Columns.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="32">
   <si>
     <t xml:space="preserve">PIT_ID</t>
   </si>
@@ -84,6 +84,21 @@
   </si>
   <si>
     <t xml:space="preserve">P20000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montipora aequituberculata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2024Oct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T03</t>
   </si>
   <si>
     <t xml:space="preserve">NAME</t>
@@ -185,7 +200,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -208,6 +223,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -333,13 +352,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="23.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.81"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -526,6 +545,57 @@
         <v>7</v>
       </c>
       <c r="E12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>45595</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>45580</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>45595</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>45580</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>45595</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>45580</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -552,7 +622,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -562,7 +632,7 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -572,12 +642,12 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -587,12 +657,12 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>